<commit_message>
Add battery register sheet with real location/quantity/type data
New sheet "سجل البطاريات حسب الموقع" combines two lists the user
provided (a photographed 36-location table and a follow-up 37-item
list), 73 rows total, dates omitted per request. Locations appearing
in both lists are kept as separate rows rather than merged, since
their battery type/count differ and there's no evidence they're the
same physical batteries.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XZ2ZP3nr7izgaJQSr6bH1E
</commit_message>
<xml_diff>
--- a/ups-database/UPS_Battery_Orders_2025.xlsx
+++ b/ups-database/UPS_Battery_Orders_2025.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="طلبات البطاريات 2025" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="سجل البطاريات حسب الموقع" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="طلبات البطاريات 2025" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,8 +74,13 @@
       <color rgb="00000000"/>
       <sz val="10.5"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A2433"/>
+      <sz val="10.5"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -99,6 +105,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF9DB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAFBFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -128,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -165,6 +176,24 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -554,6 +583,1493 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E78"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>سجل بطاريات أجهزة الـ UPS حسب الموقع</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>مجمّع من قائمتين زوّد بهما المستخدم (جدول مصوَّر + قائمة مرقّمة). لا تواريخ - كما طُلب.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>إجمالي عدد البطاريات</t>
+        </is>
+      </c>
+      <c r="E3" s="4">
+        <f>SUM(C6:C78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>عدد المواقع</t>
+        </is>
+      </c>
+      <c r="E4" s="3">
+        <f>COUNTA(B6:B78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>الموقع</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>العدد</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>نوع/سعة البطارية</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>ملاحظات</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات بمحوت</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>12V 26AH</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>مهام الدقم</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>12V 26AH</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>توقيف الداخلية</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>240</v>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>الأحوال المدنية السيب المبنى رقم 2</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>12V 65AH</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>مركز شرطة الوطية الطابق الأرضي والطابق الأول</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>12V 40AH</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>مهام الخوض الدور الثاني</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>12V 42AH</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>مركز شرطة سمائل</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>12V 40AH</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة ضنك</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>76</v>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>12V 40AH</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>مركز شرطة صلالة الدور الأرضي</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>12V 26AH</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة الكامل الدور الأرضي</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>12V 65AH</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>مبنى الإدارة بمهام نزوى الدور الأرضي</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>12V 42AH</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>مبنى الإدارة بمهام نزوى الدور الأول</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>12V 42AH</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>مركز شرطة بهلاء</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>12V 42AH</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>مركز خطمة ملاحة</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="n">
+        <v>240</v>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات بصحم</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات بسمائل</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="n">
+        <v>80</v>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات جعلان بني بو علي</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="n">
+        <v>96</v>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>عيادة مهام نزوى</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>12V 26AH</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات بإزكي</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>12V 42AH</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة السويق</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="n">
+        <v>29</v>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>12V 102AH</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات بالقرم</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>12V 42AH</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات بالدقم (الجوازات 1)</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>12V 55AH</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات نخل</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E28" s="16" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>عيادة مهام السليل</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>12V 26AH</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>عيادة الخيالة بالوطية</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>12V 150AH</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>مبنى التحريات بقيادة مسقط</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>12V 42AH</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>منفذ حماسة</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E32" s="16" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة صحار</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>12V 42AH</t>
+        </is>
+      </c>
+      <c r="E33" s="18" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>عيادة مهام صور</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E34" s="16" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="B35" s="18" t="inlineStr">
+        <is>
+          <t>مبنى الإدارة بمهام عبري</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>12V 42AH</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>مركز شرطة الدقم</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="n">
+        <v>28</v>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>12V 55AH</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة محوت</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>12V 65AH</t>
+        </is>
+      </c>
+      <c r="E37" s="18" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>مبنى تحريات الدقم</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="n">
+        <v>42</v>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>12V 40AH</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة العذيبة الدور الأول</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>12V 42AH</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات بالدقم (الجوازات 2)</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>12V 55AH</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" s="18" t="inlineStr">
+        <is>
+          <t>الإدارة العامة للمشاريع والصيانة</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>12V 26AH</t>
+        </is>
+      </c>
+      <c r="E41" s="18" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>منفذ خطم الشكلة - الجوازات (القادمون)</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="n">
+        <v>160</v>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="n">
+        <v>38</v>
+      </c>
+      <c r="B43" s="18" t="inlineStr">
+        <is>
+          <t>منفذ حماسة (المغادرون)</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E43" s="18" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="n">
+        <v>39</v>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>إدارة التوقيف بالداخلية (التحقيق)</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" s="18" t="inlineStr">
+        <is>
+          <t>إدارة التوقيف بالداخلية (مراقبة الرجال)</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="n">
+        <v>120</v>
+      </c>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E45" s="18" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات بإزكي</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>12V 26AH</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات بالقرم الطابق الأرضي</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>12V 39.6AH</t>
+        </is>
+      </c>
+      <c r="E47" s="18" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>مركز شرطة وادي المعاول الطابق الأول</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="D48" s="15" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E48" s="16" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات بنخل</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="n">
+        <v>120</v>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E49" s="18" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="15" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>إدارة التوقيف بجنوب الباطنة (المحكمة)</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E50" s="16" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة سمائل الطابق الأرضي</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D51" s="17" t="inlineStr">
+        <is>
+          <t>12V 39.6AH</t>
+        </is>
+      </c>
+      <c r="E51" s="18" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="15" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>مركز شرطة سمائل الطابق الأول</t>
+        </is>
+      </c>
+      <c r="C52" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D52" s="15" t="inlineStr">
+        <is>
+          <t>12V 39.6AH</t>
+        </is>
+      </c>
+      <c r="E52" s="16" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة الدقم</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>12V 55AH</t>
+        </is>
+      </c>
+      <c r="E53" s="18" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="15" t="n">
+        <v>49</v>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>مبنى التحريات بالدقم</t>
+        </is>
+      </c>
+      <c r="C54" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="D54" s="15" t="inlineStr">
+        <is>
+          <t>12V 40AH</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="B55" s="18" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات بسمائل</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E55" s="18" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="15" t="n">
+        <v>51</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>مبنى خدمات الدقم الطابق الأرضي</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D56" s="15" t="inlineStr">
+        <is>
+          <t>12V 55AH</t>
+        </is>
+      </c>
+      <c r="E56" s="16" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="n">
+        <v>52</v>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
+          <t>مبنى خدمات الدقم الطابق الأول</t>
+        </is>
+      </c>
+      <c r="C57" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
+        <is>
+          <t>12V 55AH</t>
+        </is>
+      </c>
+      <c r="E57" s="18" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="15" t="n">
+        <v>53</v>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>وحدة المهام الخاصة بالدقم الطابق الأرضي</t>
+        </is>
+      </c>
+      <c r="C58" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D58" s="15" t="inlineStr">
+        <is>
+          <t>12V 26AH</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="n">
+        <v>54</v>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة محوت</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D59" s="17" t="inlineStr">
+        <is>
+          <t>12V 65AH</t>
+        </is>
+      </c>
+      <c r="E59" s="18" t="inlineStr">
+        <is>
+          <t>الجهاز (100KVA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="15" t="n">
+        <v>55</v>
+      </c>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات محوت</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D60" s="15" t="inlineStr">
+        <is>
+          <t>12V 26AH</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>تم تركيب module جديد عدد 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="n">
+        <v>56</v>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>وحدة المهام الخاصة بنزوى الطابق الأرضي</t>
+        </is>
+      </c>
+      <c r="C61" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D61" s="17" t="inlineStr">
+        <is>
+          <t>12V 39.6AH</t>
+        </is>
+      </c>
+      <c r="E61" s="18" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="15" t="n">
+        <v>57</v>
+      </c>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>وحدة المهام الخاصة بنزوى الطابق الأول</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>12V 39.6AH</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="n">
+        <v>58</v>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة بهلاء</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D63" s="17" t="inlineStr">
+        <is>
+          <t>12V 39.6AH</t>
+        </is>
+      </c>
+      <c r="E63" s="18" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="n">
+        <v>59</v>
+      </c>
+      <c r="B64" s="16" t="inlineStr">
+        <is>
+          <t>مركز شرطة الحمراء الطابق الأول</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="n">
+        <v>60</v>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>12V 26AH</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="n">
+        <v>60</v>
+      </c>
+      <c r="B65" s="18" t="inlineStr">
+        <is>
+          <t>وحدة المهام الخاصة بعبري - الإدارة الطابق الأرضي</t>
+        </is>
+      </c>
+      <c r="C65" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D65" s="17" t="inlineStr">
+        <is>
+          <t>12V 39.6AH</t>
+        </is>
+      </c>
+      <c r="E65" s="18" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="15" t="n">
+        <v>61</v>
+      </c>
+      <c r="B66" s="16" t="inlineStr">
+        <is>
+          <t>وحدة المهام الخاصة بنزوى - العيادة</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D66" s="15" t="inlineStr">
+        <is>
+          <t>12V 26AH</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="n">
+        <v>62</v>
+      </c>
+      <c r="B67" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة ضنك الطابق الأرضي</t>
+        </is>
+      </c>
+      <c r="C67" s="17" t="n">
+        <v>38</v>
+      </c>
+      <c r="D67" s="17" t="inlineStr">
+        <is>
+          <t>12V 39.6AH</t>
+        </is>
+      </c>
+      <c r="E67" s="18" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="n">
+        <v>63</v>
+      </c>
+      <c r="B68" s="16" t="inlineStr">
+        <is>
+          <t>وحدة المهام الخاصة بصور - العيادة</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="n">
+        <v>120</v>
+      </c>
+      <c r="D68" s="15" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="n">
+        <v>64</v>
+      </c>
+      <c r="B69" s="18" t="inlineStr">
+        <is>
+          <t>مبنى الخدمات جعلان بني بوعلي</t>
+        </is>
+      </c>
+      <c r="C69" s="17" t="n">
+        <v>90</v>
+      </c>
+      <c r="D69" s="17" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E69" s="18" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="15" t="n">
+        <v>65</v>
+      </c>
+      <c r="B70" s="16" t="inlineStr">
+        <is>
+          <t>مركز شرطة الكامل الطابق الأرضي</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>12V 65AH</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="17" t="n">
+        <v>66</v>
+      </c>
+      <c r="B71" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة جعلان بني بوحسن</t>
+        </is>
+      </c>
+      <c r="C71" s="17" t="n">
+        <v>80</v>
+      </c>
+      <c r="D71" s="17" t="inlineStr">
+        <is>
+          <t>12V 9AH</t>
+        </is>
+      </c>
+      <c r="E71" s="18" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="15" t="n">
+        <v>67</v>
+      </c>
+      <c r="B72" s="16" t="inlineStr">
+        <is>
+          <t>مبنى خدمات صور الطابق الأرضي</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="n">
+        <v>62</v>
+      </c>
+      <c r="D72" s="15" t="inlineStr">
+        <is>
+          <t>12V 18AH</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr">
+        <is>
+          <t>مبنى خدمات صور الطابق الأول: نقص 2 بطارية من نوع 18AH</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="17" t="n">
+        <v>68</v>
+      </c>
+      <c r="B73" s="18" t="inlineStr">
+        <is>
+          <t>وحدة المهام الخاصة بعبري الطابق الأول</t>
+        </is>
+      </c>
+      <c r="C73" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="D73" s="17" t="inlineStr">
+        <is>
+          <t>12V 26AH</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="15" t="n">
+        <v>69</v>
+      </c>
+      <c r="B74" s="16" t="inlineStr">
+        <is>
+          <t>مركز شرطة الوطية الطابق الأرضي</t>
+        </is>
+      </c>
+      <c r="C74" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>12V 39.6AH</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="B75" s="18" t="inlineStr">
+        <is>
+          <t>مركز شرطة الوطية الطابق الأول</t>
+        </is>
+      </c>
+      <c r="C75" s="17" t="n">
+        <v>29</v>
+      </c>
+      <c r="D75" s="17" t="inlineStr">
+        <is>
+          <t>12V 39.6AH</t>
+        </is>
+      </c>
+      <c r="E75" s="18" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="15" t="n">
+        <v>71</v>
+      </c>
+      <c r="B76" s="16" t="inlineStr">
+        <is>
+          <t>وحدة المهام الخاصة بالخوض الطابق الأول</t>
+        </is>
+      </c>
+      <c r="C76" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="D76" s="15" t="inlineStr">
+        <is>
+          <t>12V 39.6AH</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="17" t="n">
+        <v>72</v>
+      </c>
+      <c r="B77" s="18" t="inlineStr">
+        <is>
+          <t>مستشفى المدينة الطبية - قسم تقنية المعلومات</t>
+        </is>
+      </c>
+      <c r="C77" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="D77" s="17" t="inlineStr">
+        <is>
+          <t>12V 27AH</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="15" t="n">
+        <v>73</v>
+      </c>
+      <c r="B78" s="16" t="inlineStr">
+        <is>
+          <t>الإدارة العامة للجوازات والأحوال المدنية - مبنى الأحوال المدنية رقم 2 (الوافدين)</t>
+        </is>
+      </c>
+      <c r="C78" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="D78" s="15" t="inlineStr">
+        <is>
+          <t>12V 66AH</t>
+        </is>
+      </c>
+      <c r="E78" s="16" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>